<commit_message>
Enhance metadata processing in R script; add safe extraction function and write complete metadata to CSV
</commit_message>
<xml_diff>
--- a/eod_logger_4/Uganda_2023/Recordings_Sessions_Metadata.xlsx
+++ b/eod_logger_4/Uganda_2023/Recordings_Sessions_Metadata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefa\Seafile\Uni\01 Research Projects\04 Uganda 2023 EOD loggers\01 Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Projects\EOD_pulse_analysis\eod_logger_4\Uganda_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0853D337-EE2B-4439-B7EE-57F12B160063}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A1D4A2-6603-4022-97FE-4A3E0643B036}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="24096" windowHeight="20976" xr2:uid="{1B50041A-606E-4BAA-8BC2-5A1CB87C2F31}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="24090" windowHeight="20970" xr2:uid="{1B50041A-606E-4BAA-8BC2-5A1CB87C2F31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -539,7 +539,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -555,7 +555,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -852,17 +852,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2B4DF18-2126-4684-B12F-60ED5D48E1F2}">
   <dimension ref="A1:BE73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="47" width="8.77734375" style="4"/>
-    <col min="48" max="49" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="47" width="8.7109375" style="4"/>
+    <col min="48" max="49" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1035,7 +1036,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>34</v>
       </c>
@@ -1046,7 +1047,7 @@
         <v>45210</v>
       </c>
       <c r="D2" s="2">
-        <v>45182</v>
+        <v>45212</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>47</v>
@@ -1106,7 +1107,7 @@
       </c>
       <c r="BE2" s="1"/>
     </row>
-    <row r="3" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>34</v>
       </c>
@@ -1117,7 +1118,7 @@
         <v>45210</v>
       </c>
       <c r="D3" s="2">
-        <v>45182</v>
+        <v>45212</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>49</v>
@@ -1177,7 +1178,7 @@
       </c>
       <c r="BE3" s="1"/>
     </row>
-    <row r="4" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>34</v>
       </c>
@@ -1248,7 +1249,7 @@
       </c>
       <c r="BE4" s="1"/>
     </row>
-    <row r="5" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -1313,7 +1314,7 @@
       </c>
       <c r="BE5" s="1"/>
     </row>
-    <row r="6" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>34</v>
       </c>
@@ -1382,7 +1383,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>34</v>
       </c>
@@ -1456,7 +1457,7 @@
       </c>
       <c r="BE7" s="1"/>
     </row>
-    <row r="8" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>34</v>
       </c>
@@ -1547,7 +1548,7 @@
       </c>
       <c r="BE8" s="1"/>
     </row>
-    <row r="9" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>34</v>
       </c>
@@ -1637,7 +1638,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>34</v>
       </c>
@@ -1725,7 +1726,7 @@
       </c>
       <c r="BE10" s="1"/>
     </row>
-    <row r="11" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>34</v>
       </c>
@@ -1812,7 +1813,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>34</v>
       </c>
@@ -1893,7 +1894,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="13" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>34</v>
       </c>
@@ -1968,7 +1969,7 @@
       </c>
       <c r="BE13" s="1"/>
     </row>
-    <row r="14" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>34</v>
       </c>
@@ -2037,7 +2038,7 @@
       </c>
       <c r="BE14" s="1"/>
     </row>
-    <row r="15" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
@@ -2119,7 +2120,7 @@
       </c>
       <c r="BE15" s="1"/>
     </row>
-    <row r="16" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>34</v>
       </c>
@@ -2188,7 +2189,7 @@
       </c>
       <c r="BE16" s="1"/>
     </row>
-    <row r="17" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
@@ -2253,7 +2254,7 @@
       </c>
       <c r="BE17" s="1"/>
     </row>
-    <row r="18" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -2318,7 +2319,7 @@
       </c>
       <c r="BE18" s="1"/>
     </row>
-    <row r="19" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
@@ -2329,7 +2330,7 @@
         <v>45208</v>
       </c>
       <c r="D19" s="2">
-        <v>45180</v>
+        <v>45210</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>53</v>
@@ -2387,7 +2388,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>23</v>
       </c>
@@ -2450,7 +2451,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>23</v>
       </c>
@@ -2511,7 +2512,7 @@
       </c>
       <c r="BE21" s="1"/>
     </row>
-    <row r="22" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>23</v>
       </c>
@@ -2574,7 +2575,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
@@ -2635,7 +2636,7 @@
       </c>
       <c r="BE23" s="1"/>
     </row>
-    <row r="24" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
@@ -2698,7 +2699,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -2761,7 +2762,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>23</v>
       </c>
@@ -2824,7 +2825,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>23</v>
       </c>
@@ -2896,7 +2897,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>23</v>
       </c>
@@ -2959,7 +2960,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>23</v>
       </c>
@@ -3022,7 +3023,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>23</v>
       </c>
@@ -3083,7 +3084,7 @@
       </c>
       <c r="BE30" s="1"/>
     </row>
-    <row r="31" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>23</v>
       </c>
@@ -3144,7 +3145,7 @@
       </c>
       <c r="BE31" s="1"/>
     </row>
-    <row r="32" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>23</v>
       </c>
@@ -3205,7 +3206,7 @@
       </c>
       <c r="BE32" s="1"/>
     </row>
-    <row r="33" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>23</v>
       </c>
@@ -3268,7 +3269,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="34" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>23</v>
       </c>
@@ -3329,7 +3330,7 @@
       </c>
       <c r="BE34" s="1"/>
     </row>
-    <row r="35" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>23</v>
       </c>
@@ -3393,7 +3394,7 @@
       </c>
       <c r="BE35" s="1"/>
     </row>
-    <row r="36" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>23</v>
       </c>
@@ -3454,7 +3455,7 @@
       </c>
       <c r="BE36" s="1"/>
     </row>
-    <row r="37" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>23</v>
       </c>
@@ -3515,7 +3516,7 @@
       </c>
       <c r="BE37" s="1"/>
     </row>
-    <row r="38" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>23</v>
       </c>
@@ -3576,7 +3577,7 @@
       </c>
       <c r="BE38" s="1"/>
     </row>
-    <row r="39" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>12</v>
       </c>
@@ -3640,7 +3641,7 @@
       </c>
       <c r="BE39" s="1"/>
     </row>
-    <row r="40" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>12</v>
       </c>
@@ -3704,7 +3705,7 @@
       </c>
       <c r="BE40" s="1"/>
     </row>
-    <row r="41" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>12</v>
       </c>
@@ -3768,7 +3769,7 @@
       </c>
       <c r="BE41" s="1"/>
     </row>
-    <row r="42" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>12</v>
       </c>
@@ -3832,7 +3833,7 @@
       </c>
       <c r="BE42" s="1"/>
     </row>
-    <row r="43" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>12</v>
       </c>
@@ -3896,7 +3897,7 @@
       </c>
       <c r="BE43" s="1"/>
     </row>
-    <row r="44" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>12</v>
       </c>
@@ -3962,7 +3963,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>12</v>
       </c>
@@ -4026,7 +4027,7 @@
       </c>
       <c r="BE45" s="1"/>
     </row>
-    <row r="46" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>12</v>
       </c>
@@ -4092,7 +4093,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>12</v>
       </c>
@@ -4158,7 +4159,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>12</v>
       </c>
@@ -4224,7 +4225,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>12</v>
       </c>
@@ -4290,7 +4291,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>12</v>
       </c>
@@ -4354,7 +4355,7 @@
       </c>
       <c r="BE50" s="1"/>
     </row>
-    <row r="51" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>12</v>
       </c>
@@ -4418,7 +4419,7 @@
       </c>
       <c r="BE51" s="1"/>
     </row>
-    <row r="52" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>12</v>
       </c>
@@ -4479,7 +4480,7 @@
       </c>
       <c r="BE52" s="1"/>
     </row>
-    <row r="53" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>12</v>
       </c>
@@ -4542,7 +4543,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="54" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>12</v>
       </c>
@@ -4603,7 +4604,7 @@
       </c>
       <c r="BE54" s="1"/>
     </row>
-    <row r="55" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>12</v>
       </c>
@@ -4664,7 +4665,7 @@
       </c>
       <c r="BE55" s="1"/>
     </row>
-    <row r="56" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>12</v>
       </c>
@@ -4725,7 +4726,7 @@
       </c>
       <c r="BE56" s="1"/>
     </row>
-    <row r="57" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>12</v>
       </c>
@@ -4786,7 +4787,7 @@
       </c>
       <c r="BE57" s="1"/>
     </row>
-    <row r="58" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>12</v>
       </c>
@@ -4847,7 +4848,7 @@
       </c>
       <c r="BE58" s="1"/>
     </row>
-    <row r="59" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>15</v>
       </c>
@@ -4858,7 +4859,7 @@
         <v>45210</v>
       </c>
       <c r="D59" s="2">
-        <v>45182</v>
+        <v>45212</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>14</v>
@@ -4918,7 +4919,7 @@
       </c>
       <c r="BE59" s="1"/>
     </row>
-    <row r="60" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>15</v>
       </c>
@@ -4929,7 +4930,7 @@
         <v>45210</v>
       </c>
       <c r="D60" s="2">
-        <v>45182</v>
+        <v>45212</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>37</v>
@@ -4991,7 +4992,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="61" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>15</v>
       </c>
@@ -5055,7 +5056,7 @@
       </c>
       <c r="BE61" s="4"/>
     </row>
-    <row r="62" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>15</v>
       </c>
@@ -5119,7 +5120,7 @@
       </c>
       <c r="BE62" s="4"/>
     </row>
-    <row r="63" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>15</v>
       </c>
@@ -5183,7 +5184,7 @@
       </c>
       <c r="BE63" s="1"/>
     </row>
-    <row r="64" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>15</v>
       </c>
@@ -5247,7 +5248,7 @@
       </c>
       <c r="BE64" s="1"/>
     </row>
-    <row r="65" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>15</v>
       </c>
@@ -5311,7 +5312,7 @@
       </c>
       <c r="BE65" s="1"/>
     </row>
-    <row r="66" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>15</v>
       </c>
@@ -5353,7 +5354,7 @@
         <v>45232.793437499997</v>
       </c>
       <c r="AX66" s="1">
-        <f t="shared" ref="AX66:AX97" si="2">(AW66-AV66)*24</f>
+        <f t="shared" ref="AX66:AX73" si="2">(AW66-AV66)*24</f>
         <v>30.333611111040227</v>
       </c>
       <c r="AY66" s="1">
@@ -5376,7 +5377,7 @@
       </c>
       <c r="BE66" s="1"/>
     </row>
-    <row r="67" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>15</v>
       </c>
@@ -5440,7 +5441,7 @@
       </c>
       <c r="BE67" s="1"/>
     </row>
-    <row r="68" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>15</v>
       </c>
@@ -5504,7 +5505,7 @@
       </c>
       <c r="BE68" s="1"/>
     </row>
-    <row r="69" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>15</v>
       </c>
@@ -5570,7 +5571,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="70" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>15</v>
       </c>
@@ -5634,7 +5635,7 @@
       </c>
       <c r="BE70" s="1"/>
     </row>
-    <row r="71" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>15</v>
       </c>
@@ -5700,7 +5701,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="72" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>15</v>
       </c>
@@ -5764,7 +5765,7 @@
       </c>
       <c r="BE72" s="1"/>
     </row>
-    <row r="73" spans="1:57" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>15</v>
       </c>

</xml_diff>